<commit_message>
Ammonia figures on NH3-FINAL-1.2: annotations from the 1.2 files, renders, manifests, ED Source Data
- fig1: the remaining typed annotations (off-scale Ag/Au values, top-3 rho) read from the tables
- fig2 (manuscript Fig. 3): median of panel h to two decimals as in the caption (5.46; min 1.995 as in
  the main text); assert P(C_Fe < C_Ru) = 1 behind the 5,000 / 5,000 label
- fig3: make_strict_lifecycle_panel.py reads the 1.2 strict-scaling outputs and prints their values
- F03 renderer: median gap to two decimals; F03_CAPTION.md on the 1.2 values
- FIG3_RENDER_SHA256.txt rebuilt on the 1.2 inputs; the Fig. 3 and F03/F10 render workflows list the
  1.2 inputs; -text rules for the 1.2 files the manifests hash
- Source Data: SourceData_EDFig2/5/6/7 rebuilt on the 1.2 tables (main-figure and methanol workbooks
  unchanged in content, kept as committed)
- figure READMEs: ammonia sources and values on 1.2

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/SourceData_EDFig5.xlsx
+++ b/source_data/SourceData_EDFig5.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>analysis/nh3_supported_2026_10_06/supported_candidates.csv (status primary*, cost present); rate per g metal = rate per g catalyst / metal content (fused Fe 71.51 wt%, run_supported_chain.py); Fe benchmark analysis/nh3_supported_2026_10_06/summary.json</t>
+          <t>analysis/nh3_supported_2026_10_06/nh3_1_2/supported_candidates.csv (status primary*, cost present); rate per g metal = rate per g catalyst / metal content (fused Fe 71.51 wt%, run_supported_chain.py); Fe benchmark analysis/nh3_supported_2026_10_06/nh3_1_2/summary.json</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>analysis/nh3_supported_2026_10_06/supported_candidates.csv</t>
+          <t>analysis/nh3_supported_2026_10_06/nh3_1_2/supported_candidates.csv</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -513,7 +513,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>analysis/nh3_supported_2026_10_06/supported_candidates.csv (lowest cost per metal; checked against summary.json per_metal)</t>
+          <t>analysis/nh3_supported_2026_10_06/nh3_1_2/supported_candidates.csv (lowest cost per metal; checked against summary.json per_metal)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -531,7 +531,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>analysis/nh3_supported_2026_10_06/supported_candidates.csv</t>
+          <t>analysis/nh3_supported_2026_10_06/nh3_1_2/supported_candidates.csv</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>source: analysis/nh3_supported_2026_10_06/supported_candidates.csv (status primary*, cost present); rate per g metal = rate per g catalyst / metal content (fused Fe 71.51 wt%, run_supported_chain.py); Fe benchmark analysis/nh3_supported_2026_10_06/summary.json</t>
+          <t>source: analysis/nh3_supported_2026_10_06/nh3_1_2/supported_candidates.csv (status primary*, cost present); rate per g metal = rate per g catalyst / metal content (fused Fe 71.51 wt%, run_supported_chain.py); Fe benchmark analysis/nh3_supported_2026_10_06/nh3_1_2/summary.json</t>
         </is>
       </c>
     </row>
@@ -674,10 +674,10 @@
         <v>427902.3623051129</v>
       </c>
       <c r="H4" t="n">
-        <v>15.3177523999683</v>
+        <v>11.00905495490219</v>
       </c>
       <c r="I4" t="n">
-        <v>14.41663977470939</v>
+        <v>9.922677911098129</v>
       </c>
       <c r="J4" t="n">
         <v>99</v>
@@ -686,7 +686,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fe1−xO</t>
+          <t>20% Fe–BaH2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -695,31 +695,31 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>71.51000000000001</v>
+        <v>20</v>
       </c>
       <c r="D5" t="n">
-        <v>430</v>
+        <v>350</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>0.1</v>
       </c>
       <c r="F5" t="n">
-        <v>11900</v>
+        <v>384</v>
       </c>
       <c r="G5" t="n">
-        <v>16641.02922668158</v>
+        <v>1920</v>
       </c>
       <c r="H5" t="n">
-        <v>15.5091508671665</v>
+        <v>11.18641879500925</v>
       </c>
       <c r="J5" t="n">
-        <v>157</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20% Fe–BaH2</t>
+          <t>Fe1−xO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -728,25 +728,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>20</v>
+        <v>71.51000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>350</v>
+        <v>430</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>384</v>
+        <v>11900</v>
       </c>
       <c r="G6" t="n">
-        <v>1920</v>
+        <v>16641.02922668158</v>
       </c>
       <c r="H6" t="n">
-        <v>15.54287801912185</v>
+        <v>11.73700517148674</v>
       </c>
       <c r="J6" t="n">
-        <v>79</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7">
@@ -776,7 +776,7 @@
         <v>12865.33351978744</v>
       </c>
       <c r="H7" t="n">
-        <v>15.68135157201682</v>
+        <v>11.9176365622879</v>
       </c>
       <c r="J7" t="n">
         <v>157</v>
@@ -785,139 +785,139 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ru/Ba–Ca(NH2)2</t>
+          <t>10% Fe/C</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Fe</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>10</v>
       </c>
       <c r="D8" t="n">
-        <v>360</v>
+        <v>400</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>60400</v>
+        <v>14400</v>
       </c>
       <c r="G8" t="n">
-        <v>604000</v>
+        <v>144000</v>
       </c>
       <c r="H8" t="n">
-        <v>15.88075081788533</v>
-      </c>
-      <c r="I8" t="n">
-        <v>14.75844177235617</v>
+        <v>11.9766540053931</v>
       </c>
       <c r="J8" t="n">
-        <v>106</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10% Fe/C</t>
+          <t>Ru/Ba–Ca(NH2)2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Fe</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>10</v>
       </c>
       <c r="D9" t="n">
-        <v>400</v>
+        <v>360</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F9" t="n">
-        <v>14400</v>
+        <v>60400</v>
       </c>
       <c r="G9" t="n">
-        <v>144000</v>
+        <v>604000</v>
       </c>
       <c r="H9" t="n">
-        <v>16.01706713081194</v>
+        <v>12.10108825207923</v>
+      </c>
+      <c r="I9" t="n">
+        <v>10.60159008766887</v>
       </c>
       <c r="J9" t="n">
-        <v>154</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ru/Ca(NH2)2</t>
+          <t>80% Fe/Ce0.8Sm0.2O2−δ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Fe</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="D10" t="n">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>15800</v>
+        <v>8700</v>
       </c>
       <c r="G10" t="n">
-        <v>158000</v>
+        <v>10875</v>
       </c>
       <c r="H10" t="n">
-        <v>16.29624559873036</v>
-      </c>
-      <c r="I10" t="n">
-        <v>15.05550513764555</v>
+        <v>12.57145822859276</v>
       </c>
       <c r="J10" t="n">
-        <v>116</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>80% Fe/Ce0.8Sm0.2O2−δ</t>
+          <t>Ru/Ca(NH2)2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fe</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="D11" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F11" t="n">
-        <v>8700</v>
+        <v>15800</v>
       </c>
       <c r="G11" t="n">
-        <v>10875</v>
+        <v>158000</v>
       </c>
       <c r="H11" t="n">
-        <v>16.31056913453592</v>
+        <v>12.75523346684027</v>
+      </c>
+      <c r="I11" t="n">
+        <v>11.06708958692604</v>
       </c>
       <c r="J11" t="n">
-        <v>84</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12">
@@ -947,7 +947,7 @@
         <v>2735429.38895166</v>
       </c>
       <c r="H12" t="n">
-        <v>16.70435378485601</v>
+        <v>12.91816069871172</v>
       </c>
       <c r="J12" t="n">
         <v>158</v>
@@ -956,37 +956,34 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ru/AC-G</t>
+          <t>5.2 wt% Co/CNT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10</v>
+        <v>5.2</v>
       </c>
       <c r="D13" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>312500</v>
+        <v>4800</v>
       </c>
       <c r="G13" t="n">
-        <v>3125000</v>
+        <v>92307.6923076923</v>
       </c>
       <c r="H13" t="n">
-        <v>17.22165142925473</v>
-      </c>
-      <c r="I13" t="n">
-        <v>15.49738797410795</v>
+        <v>13.10040832765772</v>
       </c>
       <c r="J13" t="n">
-        <v>109</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14">
@@ -1016,10 +1013,10 @@
         <v>105000</v>
       </c>
       <c r="H14" t="n">
-        <v>17.79478561142073</v>
+        <v>13.10579423381466</v>
       </c>
       <c r="I14" t="n">
-        <v>15.62490554740077</v>
+        <v>11.35834633242901</v>
       </c>
       <c r="J14" t="n">
         <v>105</v>
@@ -1028,34 +1025,37 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5.2 wt% Co/CNT</t>
+          <t>Ru/AC-G</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5.2</v>
+        <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F15" t="n">
-        <v>4800</v>
+        <v>312500</v>
       </c>
       <c r="G15" t="n">
-        <v>92307.6923076923</v>
+        <v>3125000</v>
       </c>
       <c r="H15" t="n">
-        <v>18.27631008120813</v>
+        <v>13.75565772222116</v>
+      </c>
+      <c r="I15" t="n">
+        <v>11.92929982828479</v>
       </c>
       <c r="J15" t="n">
-        <v>199</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16">
@@ -1085,7 +1085,7 @@
         <v>566666.6666666666</v>
       </c>
       <c r="H16" t="n">
-        <v>18.9237857349846</v>
+        <v>13.96716340798016</v>
       </c>
       <c r="J16" t="n">
         <v>82</v>
@@ -1094,37 +1094,34 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ru/Ce0.5La0.5O1.75</t>
+          <t>Ni/LaN NPs</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>12.5</v>
       </c>
       <c r="D17" t="n">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F17" t="n">
-        <v>31300</v>
+        <v>2665</v>
       </c>
       <c r="G17" t="n">
-        <v>626000</v>
+        <v>21320</v>
       </c>
       <c r="H17" t="n">
-        <v>19.22956838661794</v>
-      </c>
-      <c r="I17" t="n">
-        <v>16.46737343743095</v>
+        <v>14.31774898548576</v>
       </c>
       <c r="J17" t="n">
-        <v>77</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18">
@@ -1154,10 +1151,10 @@
         <v>74000</v>
       </c>
       <c r="H18" t="n">
-        <v>19.52695484553665</v>
+        <v>14.36812191584121</v>
       </c>
       <c r="I18" t="n">
-        <v>16.38224917302435</v>
+        <v>12.15351523255796</v>
       </c>
       <c r="J18" t="n">
         <v>105</v>
@@ -1166,7 +1163,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ru/La2Ce2O7</t>
+          <t>Ru/Ce0.5La0.5O1.75</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1175,112 +1172,112 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D19" t="n">
-        <v>425</v>
+        <v>350</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>52700</v>
+        <v>31300</v>
       </c>
       <c r="G19" t="n">
-        <v>1317500</v>
+        <v>626000</v>
       </c>
       <c r="H19" t="n">
-        <v>19.89232403784026</v>
+        <v>14.49620887516304</v>
       </c>
       <c r="I19" t="n">
-        <v>17.21686732491621</v>
+        <v>12.48171787392431</v>
       </c>
       <c r="J19" t="n">
-        <v>193</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1% Fe/BaTiO3−xHx</t>
+          <t>Ru/La0.5Pr0.5O1.75</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Fe</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
         <v>400</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>14000</v>
+        <v>60200</v>
       </c>
       <c r="G20" t="n">
-        <v>1400000</v>
+        <v>1204000</v>
       </c>
       <c r="H20" t="n">
-        <v>19.93945101197486</v>
+        <v>14.91238342733496</v>
+      </c>
+      <c r="I20" t="n">
+        <v>12.72332798872948</v>
       </c>
       <c r="J20" t="n">
-        <v>81</v>
+        <v>176</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ru/La0.5Pr0.5O1.75</t>
+          <t>1% Fe/BaTiO3−xHx</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Fe</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
         <v>400</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F21" t="n">
-        <v>60200</v>
+        <v>14000</v>
       </c>
       <c r="G21" t="n">
-        <v>1204000</v>
+        <v>1400000</v>
       </c>
       <c r="H21" t="n">
-        <v>20.15445709110676</v>
-      </c>
-      <c r="I21" t="n">
-        <v>17.11781261270464</v>
+        <v>14.92613380711864</v>
       </c>
       <c r="J21" t="n">
-        <v>176</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ni/LaN NPs</t>
+          <t>Ru/HT-C12A7:e−</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>12.5</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
         <v>340</v>
@@ -1289,22 +1286,25 @@
         <v>0.1</v>
       </c>
       <c r="F22" t="n">
-        <v>2665</v>
+        <v>2290</v>
       </c>
       <c r="G22" t="n">
-        <v>21320</v>
+        <v>114500</v>
       </c>
       <c r="H22" t="n">
-        <v>20.41458137591642</v>
+        <v>15.09099472295203</v>
+      </c>
+      <c r="I22" t="n">
+        <v>12.9810159426842</v>
       </c>
       <c r="J22" t="n">
-        <v>134</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ru/HT-C12A7:e−</t>
+          <t>Ru/Ca(NH2)2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="D23" t="n">
         <v>340</v>
@@ -1322,19 +1322,19 @@
         <v>0.1</v>
       </c>
       <c r="F23" t="n">
-        <v>2290</v>
+        <v>3386</v>
       </c>
       <c r="G23" t="n">
-        <v>114500</v>
+        <v>188111.1111111111</v>
       </c>
       <c r="H23" t="n">
-        <v>20.49242064997426</v>
+        <v>15.17023226255933</v>
       </c>
       <c r="I23" t="n">
-        <v>17.99470055418258</v>
+        <v>13.08215191765912</v>
       </c>
       <c r="J23" t="n">
-        <v>96</v>
+        <v>195</v>
       </c>
     </row>
     <row r="24">
@@ -1364,10 +1364,10 @@
         <v>188111.1111111111</v>
       </c>
       <c r="H24" t="n">
-        <v>20.60035403289035</v>
+        <v>15.17023226255933</v>
       </c>
       <c r="I24" t="n">
-        <v>18.17996532532548</v>
+        <v>13.08215191765912</v>
       </c>
       <c r="J24" t="n">
         <v>115</v>
@@ -1376,7 +1376,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ru/Ca(NH2)2</t>
+          <t>Ru/MgO–MIL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1385,34 +1385,34 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.8</v>
+        <v>3.1</v>
       </c>
       <c r="D25" t="n">
-        <v>340</v>
+        <v>400</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>3386</v>
+        <v>22290</v>
       </c>
       <c r="G25" t="n">
-        <v>188111.1111111111</v>
+        <v>719032.2580645161</v>
       </c>
       <c r="H25" t="n">
-        <v>20.60035403289035</v>
+        <v>15.37153204219083</v>
       </c>
       <c r="I25" t="n">
-        <v>18.17996532532548</v>
+        <v>13.15864069151495</v>
       </c>
       <c r="J25" t="n">
-        <v>195</v>
+        <v>177</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ru/MgO–MIL</t>
+          <t>Ru/La2Ce2O7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1421,67 +1421,70 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>400</v>
+        <v>425</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>22290</v>
+        <v>52700</v>
       </c>
       <c r="G26" t="n">
-        <v>719032.2580645161</v>
+        <v>1317500</v>
       </c>
       <c r="H26" t="n">
-        <v>20.78271547037707</v>
+        <v>15.61027658611987</v>
       </c>
       <c r="I26" t="n">
-        <v>17.93177808701002</v>
+        <v>13.40078220789764</v>
       </c>
       <c r="J26" t="n">
-        <v>177</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2.8% Fe/γ-Al2O3</t>
+          <t>Ru/BaCeO3−xHyNz (after 20 h)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fe</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2.8</v>
+        <v>4.5</v>
       </c>
       <c r="D27" t="n">
-        <v>320</v>
+        <v>400</v>
       </c>
       <c r="E27" t="n">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="F27" t="n">
-        <v>0.12</v>
+        <v>28570</v>
       </c>
       <c r="G27" t="n">
-        <v>4.285714285714286</v>
+        <v>634888.8888888889</v>
       </c>
       <c r="H27" t="n">
-        <v>21.2401571660666</v>
+        <v>15.76878465397993</v>
+      </c>
+      <c r="I27" t="n">
+        <v>13.30896149767969</v>
       </c>
       <c r="J27" t="n">
-        <v>67</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ru/BaCeO3−xHyNz (after 20 h)</t>
+          <t>Ru/Pr2O3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1490,70 +1493,67 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="D28" t="n">
         <v>400</v>
       </c>
       <c r="E28" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>28570</v>
+        <v>19000</v>
       </c>
       <c r="G28" t="n">
-        <v>634888.8888888889</v>
+        <v>380000</v>
       </c>
       <c r="H28" t="n">
-        <v>21.30442019260907</v>
+        <v>15.83396527488749</v>
       </c>
       <c r="I28" t="n">
-        <v>18.10680560829568</v>
+        <v>13.33477050040895</v>
       </c>
       <c r="J28" t="n">
-        <v>82</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ru/Pr2O3</t>
+          <t>3.4 wt% Co–N–C</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>3.73</v>
       </c>
       <c r="D29" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>19000</v>
+        <v>4340</v>
       </c>
       <c r="G29" t="n">
-        <v>380000</v>
+        <v>116353.8873994638</v>
       </c>
       <c r="H29" t="n">
-        <v>21.37188136664816</v>
-      </c>
-      <c r="I29" t="n">
-        <v>18.09852931446574</v>
+        <v>16.47965021363143</v>
       </c>
       <c r="J29" t="n">
-        <v>171</v>
+        <v>200</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ru/mesoporous carbon(MPC)-18</t>
+          <t>Ru/Y5Si3 NP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1562,34 +1562,34 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>13.8</v>
+        <v>10</v>
       </c>
       <c r="D30" t="n">
-        <v>360</v>
+        <v>340</v>
       </c>
       <c r="E30" t="n">
-        <v>0.99</v>
+        <v>0.1</v>
       </c>
       <c r="F30" t="n">
-        <v>10200</v>
+        <v>4448</v>
       </c>
       <c r="G30" t="n">
-        <v>73913.04347826086</v>
+        <v>44480</v>
       </c>
       <c r="H30" t="n">
-        <v>21.52722858354669</v>
+        <v>16.51471139983438</v>
       </c>
       <c r="I30" t="n">
-        <v>18.22593428354077</v>
+        <v>13.47532571003271</v>
       </c>
       <c r="J30" t="n">
-        <v>168</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ru/MPC</t>
+          <t>Ru/Y5Si3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1598,34 +1598,34 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>10</v>
+        <v>7.8</v>
       </c>
       <c r="D31" t="n">
-        <v>370</v>
+        <v>400</v>
       </c>
       <c r="E31" t="n">
-        <v>0.99</v>
+        <v>0.1</v>
       </c>
       <c r="F31" t="n">
-        <v>8100</v>
+        <v>1875</v>
       </c>
       <c r="G31" t="n">
-        <v>81000</v>
+        <v>24038.46153846154</v>
       </c>
       <c r="H31" t="n">
-        <v>21.62004243546474</v>
+        <v>16.54599950712559</v>
       </c>
       <c r="I31" t="n">
-        <v>18.39761294088624</v>
+        <v>13.92138931983496</v>
       </c>
       <c r="J31" t="n">
-        <v>169</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Ru/Y5Si3</t>
+          <t>Ru/Li/AC</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1634,70 +1634,67 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
       <c r="D32" t="n">
-        <v>400</v>
+        <v>460</v>
       </c>
       <c r="E32" t="n">
-        <v>0.1</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>1875</v>
+        <v>106120</v>
       </c>
       <c r="G32" t="n">
-        <v>24038.46153846154</v>
+        <v>2210833.333333333</v>
       </c>
       <c r="H32" t="n">
-        <v>21.63012599814882</v>
+        <v>16.59696432323943</v>
       </c>
       <c r="I32" t="n">
-        <v>18.48118443757064</v>
+        <v>14.09976652817094</v>
       </c>
       <c r="J32" t="n">
-        <v>117</v>
+        <v>187</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ru/MPC</t>
+          <t>2.8% Fe/γ-Al2O3</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Fe</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="D33" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="E33" t="n">
-        <v>0.99</v>
+        <v>0.1</v>
       </c>
       <c r="F33" t="n">
-        <v>10400</v>
+        <v>0.12</v>
       </c>
       <c r="G33" t="n">
-        <v>104000</v>
+        <v>4.285714285714286</v>
       </c>
       <c r="H33" t="n">
-        <v>21.64527485456869</v>
-      </c>
-      <c r="I33" t="n">
-        <v>18.41506608586634</v>
+        <v>16.60269600438175</v>
       </c>
       <c r="J33" t="n">
-        <v>170</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ru/Li/AC</t>
+          <t>Ru/Pr2O3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1706,34 +1703,34 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="D34" t="n">
-        <v>460</v>
+        <v>400</v>
       </c>
       <c r="E34" t="n">
         <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>106120</v>
+        <v>64000</v>
       </c>
       <c r="G34" t="n">
-        <v>2210833.333333333</v>
+        <v>1280000</v>
       </c>
       <c r="H34" t="n">
-        <v>21.76221947626512</v>
+        <v>16.63726398293645</v>
       </c>
       <c r="I34" t="n">
-        <v>18.8149928148991</v>
+        <v>14.1055645473568</v>
       </c>
       <c r="J34" t="n">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ru/Sibunit</t>
+          <t>Ru/mesoporous carbon(MPC)-18</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1742,70 +1739,67 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>13.8</v>
       </c>
       <c r="D35" t="n">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="E35" t="n">
-        <v>0.7</v>
+        <v>0.99</v>
       </c>
       <c r="F35" t="n">
-        <v>1540</v>
+        <v>10200</v>
       </c>
       <c r="G35" t="n">
-        <v>38500</v>
+        <v>73913.04347826086</v>
       </c>
       <c r="H35" t="n">
-        <v>21.78930735776838</v>
+        <v>16.77129437936286</v>
       </c>
       <c r="I35" t="n">
-        <v>18.98098696378628</v>
+        <v>13.89023528329446</v>
       </c>
       <c r="J35" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ru/Ti–Ce–S</t>
+          <t>Ni–LiH</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>59.5</v>
       </c>
       <c r="D36" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F36" t="n">
-        <v>14580</v>
+        <v>40</v>
       </c>
       <c r="G36" t="n">
-        <v>486000</v>
+        <v>67.22689075630252</v>
       </c>
       <c r="H36" t="n">
-        <v>21.92174435531882</v>
-      </c>
-      <c r="I36" t="n">
-        <v>19.29062764485845</v>
+        <v>16.7884915341495</v>
       </c>
       <c r="J36" t="n">
-        <v>172</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ru/Al2O3-980</t>
+          <t>Ru/Sibunit</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1814,34 +1808,34 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="F37" t="n">
-        <v>7217</v>
+        <v>1540</v>
       </c>
       <c r="G37" t="n">
-        <v>144340</v>
+        <v>38500</v>
       </c>
       <c r="H37" t="n">
-        <v>21.98536682360781</v>
+        <v>16.78895506532469</v>
       </c>
       <c r="I37" t="n">
-        <v>19.00547571699945</v>
+        <v>14.25501235074186</v>
       </c>
       <c r="J37" t="n">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ru/gC–Al2O3</t>
+          <t>Ru/Ti–Ce–S</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1850,7 +1844,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D38" t="n">
         <v>400</v>
@@ -1859,25 +1853,25 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>5611</v>
+        <v>14580</v>
       </c>
       <c r="G38" t="n">
-        <v>112220</v>
+        <v>486000</v>
       </c>
       <c r="H38" t="n">
-        <v>22.10515879556368</v>
+        <v>16.83787763443479</v>
       </c>
       <c r="I38" t="n">
-        <v>19.08378650055852</v>
+        <v>14.42035518741308</v>
       </c>
       <c r="J38" t="n">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ru/CeO2-r</t>
+          <t>Ru/MPC</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1886,34 +1880,34 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D39" t="n">
-        <v>400</v>
+        <v>370</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="F39" t="n">
-        <v>3830</v>
+        <v>8100</v>
       </c>
       <c r="G39" t="n">
-        <v>95750</v>
+        <v>81000</v>
       </c>
       <c r="H39" t="n">
-        <v>22.18328192693386</v>
+        <v>16.91088849309671</v>
       </c>
       <c r="I39" t="n">
-        <v>19.28841919428085</v>
+        <v>14.00262648524418</v>
       </c>
       <c r="J39" t="n">
-        <v>178</v>
+        <v>169</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ba/Ru/BN</t>
+          <t>Ru/MPC</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1922,34 +1916,34 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>4.5</v>
+        <v>10</v>
       </c>
       <c r="D40" t="n">
-        <v>400</v>
+        <v>380</v>
       </c>
       <c r="E40" t="n">
-        <v>10</v>
+        <v>0.99</v>
       </c>
       <c r="F40" t="n">
-        <v>186600</v>
+        <v>10400</v>
       </c>
       <c r="G40" t="n">
-        <v>4146666.666666667</v>
+        <v>104000</v>
       </c>
       <c r="H40" t="n">
-        <v>22.21693002558449</v>
+        <v>16.96625082693422</v>
       </c>
       <c r="I40" t="n">
-        <v>19.22566949948449</v>
+        <v>14.02324644869411</v>
       </c>
       <c r="J40" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ru/Y5Si3 NP</t>
+          <t>Ru/graphene</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1958,34 +1952,34 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>10</v>
+        <v>1.4</v>
       </c>
       <c r="D41" t="n">
-        <v>340</v>
+        <v>400</v>
       </c>
       <c r="E41" t="n">
         <v>0.1</v>
       </c>
       <c r="F41" t="n">
-        <v>4448</v>
+        <v>336</v>
       </c>
       <c r="G41" t="n">
-        <v>44480</v>
+        <v>24000</v>
       </c>
       <c r="H41" t="n">
-        <v>22.23441804576935</v>
+        <v>17.05159250202018</v>
       </c>
       <c r="I41" t="n">
-        <v>18.38651705441137</v>
+        <v>15.04490946301635</v>
       </c>
       <c r="J41" t="n">
-        <v>118</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ru/CeO2–C12H29NO (TPAOH)</t>
+          <t>Ru/HT–C12A7</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1994,34 +1988,34 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>0.1</v>
       </c>
       <c r="F42" t="n">
-        <v>32000</v>
+        <v>3050</v>
       </c>
       <c r="G42" t="n">
-        <v>1280000</v>
+        <v>152500</v>
       </c>
       <c r="H42" t="n">
-        <v>22.26949764505553</v>
+        <v>17.13907664592239</v>
       </c>
       <c r="I42" t="n">
-        <v>19.71360341245012</v>
+        <v>14.84517592806065</v>
       </c>
       <c r="J42" t="n">
-        <v>185</v>
+        <v>162</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ru@CeO2-9</t>
+          <t>Ru/BaCeO2-a</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2030,34 +2024,34 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2.48</v>
+        <v>1.25</v>
       </c>
       <c r="D43" t="n">
-        <v>425</v>
+        <v>450</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
-        <v>8500</v>
+        <v>28000</v>
       </c>
       <c r="G43" t="n">
-        <v>342741.935483871</v>
+        <v>2240000</v>
       </c>
       <c r="H43" t="n">
-        <v>22.34629490641281</v>
+        <v>17.29390925767541</v>
       </c>
       <c r="I43" t="n">
-        <v>19.77644633535914</v>
+        <v>15.26082530877137</v>
       </c>
       <c r="J43" t="n">
-        <v>101</v>
+        <v>184</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ba/Ru/Graphitic Nanofilaments (GNFS)</t>
+          <t>Ru/Al2O3-980</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2066,70 +2060,67 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D44" t="n">
         <v>400</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>18570</v>
+        <v>7217</v>
       </c>
       <c r="G44" t="n">
-        <v>464250</v>
+        <v>144340</v>
       </c>
       <c r="H44" t="n">
-        <v>22.401891205133</v>
+        <v>17.39025709188489</v>
       </c>
       <c r="I44" t="n">
-        <v>19.41897404157888</v>
+        <v>14.39767518403733</v>
       </c>
       <c r="J44" t="n">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ru/graphene</t>
+          <t>Ni–BaH2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1.4</v>
+        <v>20</v>
       </c>
       <c r="D45" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E45" t="n">
         <v>0.1</v>
       </c>
       <c r="F45" t="n">
-        <v>336</v>
+        <v>48</v>
       </c>
       <c r="G45" t="n">
-        <v>24000</v>
+        <v>240</v>
       </c>
       <c r="H45" t="n">
-        <v>22.42438620103372</v>
-      </c>
-      <c r="I45" t="n">
-        <v>20.2683867945907</v>
+        <v>17.40367576921054</v>
       </c>
       <c r="J45" t="n">
-        <v>165</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Ru/MC</t>
+          <t>Ru/CeO2–C12H29NO (TPAOH)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2138,34 +2129,34 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="D46" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="E46" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
-        <v>133000</v>
+        <v>32000</v>
       </c>
       <c r="G46" t="n">
-        <v>5782608.695652174</v>
+        <v>1280000</v>
       </c>
       <c r="H46" t="n">
-        <v>22.43766932192126</v>
+        <v>17.42380919718144</v>
       </c>
       <c r="I46" t="n">
-        <v>19.90059826136212</v>
+        <v>14.78631712734077</v>
       </c>
       <c r="J46" t="n">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ru/Pr2O3</t>
+          <t>Ru@CeO2-9</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2174,103 +2165,103 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>5</v>
+        <v>2.48</v>
       </c>
       <c r="D47" t="n">
-        <v>400</v>
+        <v>425</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>64000</v>
+        <v>8500</v>
       </c>
       <c r="G47" t="n">
-        <v>1280000</v>
+        <v>342741.935483871</v>
       </c>
       <c r="H47" t="n">
-        <v>22.50875227002852</v>
+        <v>17.55898712578093</v>
       </c>
       <c r="I47" t="n">
-        <v>19.11011498891022</v>
+        <v>14.84968308942984</v>
       </c>
       <c r="J47" t="n">
-        <v>182</v>
+        <v>101</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>3.4 wt% Co–N–C</t>
+          <t>Ru/BaTiO2.5H0.5</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3.73</v>
+        <v>0.86</v>
       </c>
       <c r="D48" t="n">
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
-        <v>4340</v>
+        <v>28200</v>
       </c>
       <c r="G48" t="n">
-        <v>116353.8873994638</v>
+        <v>3279069.76744186</v>
       </c>
       <c r="H48" t="n">
-        <v>22.54368102061514</v>
+        <v>17.58603666930462</v>
+      </c>
+      <c r="I48" t="n">
+        <v>15.76602252379288</v>
       </c>
       <c r="J48" t="n">
-        <v>200</v>
+        <v>81</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ru/BaCeO2-a</t>
+          <t>10 wt% Co/CeO2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1.25</v>
+        <v>10</v>
       </c>
       <c r="D49" t="n">
-        <v>450</v>
+        <v>430</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F49" t="n">
-        <v>28000</v>
+        <v>86000</v>
       </c>
       <c r="G49" t="n">
-        <v>2240000</v>
+        <v>860000</v>
       </c>
       <c r="H49" t="n">
-        <v>22.58972546066001</v>
-      </c>
-      <c r="I49" t="n">
-        <v>20.51610109982357</v>
+        <v>17.60718476082238</v>
       </c>
       <c r="J49" t="n">
-        <v>184</v>
+        <v>206</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ru/CeO2–CS</t>
+          <t>Ru/gC–Al2O3</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2279,34 +2270,34 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="D50" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>27000</v>
+        <v>5611</v>
       </c>
       <c r="G50" t="n">
-        <v>1080000</v>
+        <v>112220</v>
       </c>
       <c r="H50" t="n">
-        <v>22.63422190250466</v>
+        <v>17.62477061657694</v>
       </c>
       <c r="I50" t="n">
-        <v>19.97839032758582</v>
+        <v>14.48050159525516</v>
       </c>
       <c r="J50" t="n">
-        <v>186</v>
+        <v>174</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ru/HT–C12A7</t>
+          <t>Ru/CeO2-r</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2315,34 +2306,34 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D51" t="n">
         <v>400</v>
       </c>
       <c r="E51" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>3050</v>
+        <v>3830</v>
       </c>
       <c r="G51" t="n">
-        <v>152500</v>
+        <v>95750</v>
       </c>
       <c r="H51" t="n">
-        <v>22.73911866181321</v>
+        <v>17.63943186785973</v>
       </c>
       <c r="I51" t="n">
-        <v>20.06350601417598</v>
+        <v>14.59291070941218</v>
       </c>
       <c r="J51" t="n">
-        <v>162</v>
+        <v>178</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ru–N–mesoporous carbon (MC)</t>
+          <t>Ru/MC</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2351,7 +2342,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3.75</v>
+        <v>2.3</v>
       </c>
       <c r="D52" t="n">
         <v>400</v>
@@ -2360,94 +2351,94 @@
         <v>10</v>
       </c>
       <c r="F52" t="n">
-        <v>79000</v>
+        <v>133000</v>
       </c>
       <c r="G52" t="n">
-        <v>2106666.666666667</v>
+        <v>5782608.695652174</v>
       </c>
       <c r="H52" t="n">
-        <v>22.79707615469821</v>
+        <v>17.78793907638038</v>
       </c>
       <c r="I52" t="n">
-        <v>19.67121736144116</v>
+        <v>14.99452490188818</v>
       </c>
       <c r="J52" t="n">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Ru/BaTiO2.5H0.5</t>
+          <t>Ni/LaN bulk</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.86</v>
+        <v>5</v>
       </c>
       <c r="D53" t="n">
-        <v>400</v>
+        <v>340</v>
       </c>
       <c r="E53" t="n">
-        <v>5</v>
+        <v>0.1</v>
       </c>
       <c r="F53" t="n">
-        <v>28200</v>
+        <v>820</v>
       </c>
       <c r="G53" t="n">
-        <v>3279069.76744186</v>
+        <v>16400</v>
       </c>
       <c r="H53" t="n">
-        <v>22.97505023442373</v>
-      </c>
-      <c r="I53" t="n">
-        <v>21.13842463633245</v>
+        <v>17.84270818984833</v>
       </c>
       <c r="J53" t="n">
-        <v>81</v>
+        <v>134</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Ni–LiH</t>
+          <t>Ru/BaZrO3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>59.5</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="E54" t="n">
         <v>0.1</v>
       </c>
       <c r="F54" t="n">
-        <v>40</v>
+        <v>3630</v>
       </c>
       <c r="G54" t="n">
-        <v>67.22689075630252</v>
+        <v>181500</v>
       </c>
       <c r="H54" t="n">
-        <v>23.08299349565035</v>
+        <v>17.88596281214117</v>
+      </c>
+      <c r="I54" t="n">
+        <v>15.32170107361506</v>
       </c>
       <c r="J54" t="n">
-        <v>76</v>
+        <v>164</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ru/BaCeO3</t>
+          <t>Ba/Ru/BN</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2456,34 +2447,34 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="D55" t="n">
         <v>400</v>
       </c>
       <c r="E55" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F55" t="n">
-        <v>6450</v>
+        <v>186600</v>
       </c>
       <c r="G55" t="n">
-        <v>215000</v>
+        <v>4146666.666666667</v>
       </c>
       <c r="H55" t="n">
-        <v>23.20436073707794</v>
+        <v>17.90292095901326</v>
       </c>
       <c r="I55" t="n">
-        <v>20.12072416313562</v>
+        <v>14.62892695550267</v>
       </c>
       <c r="J55" t="n">
-        <v>181</v>
+        <v>190</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ru/BaZrO3</t>
+          <t>Ru/Yittria Stabilized Zirconia (YSZ)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2492,34 +2483,34 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="D56" t="n">
         <v>400</v>
       </c>
       <c r="E56" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>3630</v>
+        <v>5640</v>
       </c>
       <c r="G56" t="n">
-        <v>181500</v>
+        <v>1410000</v>
       </c>
       <c r="H56" t="n">
-        <v>23.22687763512296</v>
+        <v>17.96158057299256</v>
       </c>
       <c r="I56" t="n">
-        <v>20.46935647932307</v>
+        <v>16.7417116094522</v>
       </c>
       <c r="J56" t="n">
-        <v>164</v>
+        <v>173</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ru/CeO2-c</t>
+          <t>Ru/CeO2–CS</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2528,34 +2519,34 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="D57" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
-        <v>1289</v>
+        <v>27000</v>
       </c>
       <c r="G57" t="n">
-        <v>32225</v>
+        <v>1080000</v>
       </c>
       <c r="H57" t="n">
-        <v>23.22776998802789</v>
+        <v>18.0683817293354</v>
       </c>
       <c r="I57" t="n">
-        <v>19.81687091043289</v>
+        <v>15.05075190634503</v>
       </c>
       <c r="J57" t="n">
-        <v>178</v>
+        <v>186</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ru/MgO</t>
+          <t>Ba/Ru/Graphitic Nanofilaments (GNFS)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2564,34 +2555,34 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
         <v>400</v>
       </c>
       <c r="E58" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="F58" t="n">
-        <v>4200</v>
+        <v>18570</v>
       </c>
       <c r="G58" t="n">
-        <v>210000</v>
+        <v>464250</v>
       </c>
       <c r="H58" t="n">
-        <v>23.30580558092457</v>
+        <v>18.09670988494057</v>
       </c>
       <c r="I58" t="n">
-        <v>20.68866835664272</v>
+        <v>14.75551086050876</v>
       </c>
       <c r="J58" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ru/BaTiO3</t>
+          <t>Ru–N–mesoporous carbon (MC)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2600,34 +2591,34 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="D59" t="n">
         <v>400</v>
       </c>
       <c r="E59" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F59" t="n">
-        <v>15670</v>
+        <v>79000</v>
       </c>
       <c r="G59" t="n">
-        <v>391750</v>
+        <v>2106666.666666667</v>
       </c>
       <c r="H59" t="n">
-        <v>23.32917066895267</v>
+        <v>18.62326716395099</v>
       </c>
       <c r="I59" t="n">
-        <v>19.86696646925644</v>
+        <v>15.06559969859407</v>
       </c>
       <c r="J59" t="n">
-        <v>94</v>
+        <v>191</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Ru/Y–layered double oxide (LDO)</t>
+          <t>Ru/MgO</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2636,34 +2627,34 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3.85</v>
+        <v>2</v>
       </c>
       <c r="D60" t="n">
-        <v>425</v>
+        <v>400</v>
       </c>
       <c r="E60" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="F60" t="n">
-        <v>16120</v>
+        <v>4200</v>
       </c>
       <c r="G60" t="n">
-        <v>418701.2987012987</v>
+        <v>210000</v>
       </c>
       <c r="H60" t="n">
-        <v>23.37988813206525</v>
+        <v>18.82620010731137</v>
       </c>
       <c r="I60" t="n">
-        <v>19.93127182313833</v>
+        <v>15.66550940251583</v>
       </c>
       <c r="J60" t="n">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ru/MgAl–LDO</t>
+          <t>Ru/BaCeO3</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2672,34 +2663,34 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3.86</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>425</v>
+        <v>400</v>
       </c>
       <c r="E61" t="n">
         <v>3</v>
       </c>
       <c r="F61" t="n">
-        <v>14760</v>
+        <v>6450</v>
       </c>
       <c r="G61" t="n">
-        <v>382383.4196891192</v>
+        <v>215000</v>
       </c>
       <c r="H61" t="n">
-        <v>23.49895488665815</v>
+        <v>18.93939769270342</v>
       </c>
       <c r="I61" t="n">
-        <v>19.98643144807416</v>
+        <v>15.38888812365735</v>
       </c>
       <c r="J61" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Ru/CeO2–MS</t>
+          <t>Ru/CeO2-c</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2708,67 +2699,70 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="D62" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="E62" t="n">
-        <v>3.8</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>24000</v>
+        <v>1289</v>
       </c>
       <c r="G62" t="n">
-        <v>960000</v>
+        <v>32225</v>
       </c>
       <c r="H62" t="n">
-        <v>23.51767409881526</v>
+        <v>19.02352709184257</v>
       </c>
       <c r="I62" t="n">
-        <v>20.51356024600929</v>
+        <v>15.23680420967795</v>
       </c>
       <c r="J62" t="n">
-        <v>188</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Ni–BaH2</t>
+          <t>Ru/CeO2–MS</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>20</v>
+        <v>2.5</v>
       </c>
       <c r="D63" t="n">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="E63" t="n">
-        <v>0.1</v>
+        <v>3.8</v>
       </c>
       <c r="F63" t="n">
-        <v>48</v>
+        <v>24000</v>
       </c>
       <c r="G63" t="n">
-        <v>240</v>
+        <v>960000</v>
       </c>
       <c r="H63" t="n">
-        <v>23.71054935914687</v>
+        <v>19.17943173336585</v>
+      </c>
+      <c r="I63" t="n">
+        <v>15.67334591509229</v>
       </c>
       <c r="J63" t="n">
-        <v>79</v>
+        <v>188</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ru/Yittria Stabilized Zirconia (YSZ)</t>
+          <t>Ru/Y–layered double oxide (LDO)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2777,67 +2771,70 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.4</v>
+        <v>3.85</v>
       </c>
       <c r="D64" t="n">
-        <v>400</v>
+        <v>425</v>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F64" t="n">
-        <v>5640</v>
+        <v>16120</v>
       </c>
       <c r="G64" t="n">
-        <v>1410000</v>
+        <v>418701.2987012987</v>
       </c>
       <c r="H64" t="n">
-        <v>23.7109326477648</v>
+        <v>19.2233014689614</v>
       </c>
       <c r="I64" t="n">
-        <v>22.4632665502814</v>
+        <v>15.36405780006497</v>
       </c>
       <c r="J64" t="n">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>10 wt% Co/CeO2</t>
+          <t>Ru/BaTiO3</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D65" t="n">
-        <v>430</v>
+        <v>400</v>
       </c>
       <c r="E65" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F65" t="n">
-        <v>86000</v>
+        <v>15670</v>
       </c>
       <c r="G65" t="n">
-        <v>860000</v>
+        <v>391750</v>
       </c>
       <c r="H65" t="n">
-        <v>23.73387896628061</v>
+        <v>19.23517123790478</v>
+      </c>
+      <c r="I65" t="n">
+        <v>15.34505576881115</v>
       </c>
       <c r="J65" t="n">
-        <v>206</v>
+        <v>94</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Ni/LaN bulk</t>
+          <t>NI/CeN NPs</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2846,31 +2843,31 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>5</v>
+        <v>11.7</v>
       </c>
       <c r="D66" t="n">
-        <v>340</v>
+        <v>400</v>
       </c>
       <c r="E66" t="n">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="F66" t="n">
-        <v>820</v>
+        <v>6500</v>
       </c>
       <c r="G66" t="n">
-        <v>16400</v>
+        <v>55555.55555555556</v>
       </c>
       <c r="H66" t="n">
-        <v>24.08394547182962</v>
+        <v>19.28900822239036</v>
       </c>
       <c r="J66" t="n">
-        <v>134</v>
+        <v>150</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Ru/MgO</t>
+          <t>Ru/MgAl–LDO</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2879,28 +2876,28 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>4</v>
+        <v>3.86</v>
       </c>
       <c r="D67" t="n">
-        <v>400</v>
+        <v>425</v>
       </c>
       <c r="E67" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F67" t="n">
-        <v>7390</v>
+        <v>14760</v>
       </c>
       <c r="G67" t="n">
-        <v>184750</v>
+        <v>382383.4196891192</v>
       </c>
       <c r="H67" t="n">
-        <v>24.41007009522229</v>
+        <v>19.36057218899609</v>
       </c>
       <c r="I67" t="n">
-        <v>20.39998074223815</v>
+        <v>15.43516850059447</v>
       </c>
       <c r="J67" t="n">
-        <v>94</v>
+        <v>183</v>
       </c>
     </row>
     <row r="68">
@@ -2930,10 +2927,10 @@
         <v>200000</v>
       </c>
       <c r="H68" t="n">
-        <v>24.80386642961499</v>
+        <v>19.98250760663265</v>
       </c>
       <c r="I68" t="n">
-        <v>21.73392142828638</v>
+        <v>16.53186855705671</v>
       </c>
       <c r="J68" t="n">
         <v>164</v>
@@ -2942,7 +2939,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Ru/carbon nanotubes (CNT)-D</t>
+          <t>Ru/C12A7 (microcube)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2951,67 +2948,70 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
       <c r="D69" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="E69" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="F69" t="n">
-        <v>110000</v>
+        <v>5380</v>
       </c>
       <c r="G69" t="n">
-        <v>3235294.117647059</v>
+        <v>107600</v>
       </c>
       <c r="H69" t="n">
-        <v>24.9059971986012</v>
+        <v>20.18676273724735</v>
       </c>
       <c r="I69" t="n">
-        <v>20.88959536260946</v>
+        <v>16.10482926543191</v>
       </c>
       <c r="J69" t="n">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NI/CeN NPs</t>
+          <t>Ru/MgO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>11.7</v>
+        <v>4</v>
       </c>
       <c r="D70" t="n">
         <v>400</v>
       </c>
       <c r="E70" t="n">
-        <v>0.9</v>
+        <v>5</v>
       </c>
       <c r="F70" t="n">
-        <v>6500</v>
+        <v>7390</v>
       </c>
       <c r="G70" t="n">
-        <v>55555.55555555556</v>
+        <v>184750</v>
       </c>
       <c r="H70" t="n">
-        <v>25.9193907089895</v>
+        <v>20.48174255289426</v>
+      </c>
+      <c r="I70" t="n">
+        <v>16.00903266977533</v>
       </c>
       <c r="J70" t="n">
-        <v>150</v>
+        <v>94</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Ru/C12A7 (microcube)</t>
+          <t>Ru/SAs/S-1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3020,7 +3020,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>5</v>
+        <v>0.27</v>
       </c>
       <c r="D71" t="n">
         <v>400</v>
@@ -3029,61 +3029,58 @@
         <v>0.1</v>
       </c>
       <c r="F71" t="n">
-        <v>5380</v>
+        <v>1389.5</v>
       </c>
       <c r="G71" t="n">
-        <v>107600</v>
+        <v>514629.6296296296</v>
       </c>
       <c r="H71" t="n">
-        <v>26.20136441171531</v>
+        <v>20.56018708291476</v>
       </c>
       <c r="I71" t="n">
-        <v>21.9371504230411</v>
+        <v>18.95455659346021</v>
       </c>
       <c r="J71" t="n">
-        <v>196</v>
+        <v>163</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Ru/SAs/S-1</t>
+          <t>6 wt% Co/CeO2</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Ru</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>0.27</v>
+        <v>6</v>
       </c>
       <c r="D72" t="n">
-        <v>400</v>
+        <v>430</v>
       </c>
       <c r="E72" t="n">
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="F72" t="n">
-        <v>1389.5</v>
+        <v>26654</v>
       </c>
       <c r="G72" t="n">
-        <v>514629.6296296296</v>
+        <v>444233.3333333334</v>
       </c>
       <c r="H72" t="n">
-        <v>26.717317081552</v>
-      </c>
-      <c r="I72" t="n">
-        <v>25.11588950800139</v>
+        <v>20.57793051403217</v>
       </c>
       <c r="J72" t="n">
-        <v>163</v>
+        <v>205</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Ru/CeO2-r</t>
+          <t>Ru/carbon nanotubes (CNT)-D</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3092,34 +3089,34 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>10</v>
+        <v>3.4</v>
       </c>
       <c r="D73" t="n">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="E73" t="n">
         <v>10</v>
       </c>
       <c r="F73" t="n">
-        <v>115000</v>
+        <v>110000</v>
       </c>
       <c r="G73" t="n">
-        <v>1150000</v>
+        <v>3235294.117647059</v>
       </c>
       <c r="H73" t="n">
-        <v>28.11549732185807</v>
+        <v>21.05136427525452</v>
       </c>
       <c r="I73" t="n">
-        <v>22.80727609747251</v>
+        <v>16.46381976403225</v>
       </c>
       <c r="J73" t="n">
-        <v>100</v>
+        <v>194</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>6 wt% Co/CeO2</t>
+          <t>2.6 wt% Co/C12A7:e−1</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3128,58 +3125,61 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>6</v>
+        <v>2.6</v>
       </c>
       <c r="D74" t="n">
-        <v>430</v>
+        <v>400</v>
       </c>
       <c r="E74" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="F74" t="n">
-        <v>26654</v>
+        <v>1764</v>
       </c>
       <c r="G74" t="n">
-        <v>444233.3333333334</v>
+        <v>67846.15384615384</v>
       </c>
       <c r="H74" t="n">
-        <v>28.14354075398602</v>
+        <v>22.70188170215348</v>
       </c>
       <c r="J74" t="n">
-        <v>205</v>
+        <v>197</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2.6 wt% Co/C12A7:e−1</t>
+          <t>Ru/CeO2-r</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>Ru</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2.6</v>
+        <v>10</v>
       </c>
       <c r="D75" t="n">
         <v>400</v>
       </c>
       <c r="E75" t="n">
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="F75" t="n">
-        <v>1764</v>
+        <v>115000</v>
       </c>
       <c r="G75" t="n">
-        <v>67846.15384615384</v>
+        <v>1150000</v>
       </c>
       <c r="H75" t="n">
-        <v>35.13257848346144</v>
+        <v>23.53147837661924</v>
+      </c>
+      <c r="I75" t="n">
+        <v>17.6208091326523</v>
       </c>
       <c r="J75" t="n">
-        <v>197</v>
+        <v>100</v>
       </c>
     </row>
     <row r="76">
@@ -3209,10 +3209,10 @@
         <v>9750</v>
       </c>
       <c r="H76" t="n">
-        <v>41.27598549929062</v>
+        <v>37.72916488894347</v>
       </c>
       <c r="I76" t="n">
-        <v>30.30968171443131</v>
+        <v>26.26997417952612</v>
       </c>
       <c r="J76" t="n">
         <v>94</v>
@@ -3228,7 +3228,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>source: analysis/nh3_supported_2026_10_06/supported_candidates.csv</t>
+          <t>source: analysis/nh3_supported_2026_10_06/nh3_1_2/supported_candidates.csv</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>15.29170467662114</v>
+        <v>11.51578359717927</v>
       </c>
     </row>
     <row r="83">
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>17.22165142925473</v>
+        <v>13.75565772222116</v>
       </c>
     </row>
     <row r="85">
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>15.3177523999683</v>
+        <v>11.00905495490219</v>
       </c>
     </row>
     <row r="87">
@@ -3305,7 +3305,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.1242936286977958</v>
+        <v>0.2494857895223728</v>
       </c>
     </row>
     <row r="88">
@@ -3315,7 +3315,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>0.1560402943399719</v>
+        <v>0.07107045338845781</v>
       </c>
     </row>
   </sheetData>
@@ -3373,7 +3373,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>source: analysis/nh3_supported_2026_10_06/supported_candidates.csv (lowest cost per metal; checked against summary.json per_metal)</t>
+          <t>source: analysis/nh3_supported_2026_10_06/nh3_1_2/supported_candidates.csv (lowest cost per metal; checked against summary.json per_metal)</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>15.3177523999683</v>
+        <v>11.00905495490219</v>
       </c>
       <c r="D4" t="n">
         <v>54</v>
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fe1−xO</t>
+          <t>20% Fe–BaH2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15.5091508671665</v>
+        <v>11.18641879500925</v>
       </c>
       <c r="D5" t="n">
         <v>9</v>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>18.27631008120813</v>
+        <v>13.10040832765772</v>
       </c>
       <c r="D6" t="n">
         <v>5</v>
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20.41458137591642</v>
+        <v>14.31774898548576</v>
       </c>
       <c r="D7" t="n">
         <v>5</v>
@@ -3481,7 +3481,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>source: analysis/nh3_supported_2026_10_06/supported_candidates.csv</t>
+          <t>source: analysis/nh3_supported_2026_10_06/nh3_1_2/supported_candidates.csv</t>
         </is>
       </c>
     </row>
@@ -3504,7 +3504,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15.29170467662114</v>
+        <v>11.51578359717927</v>
       </c>
     </row>
   </sheetData>

</xml_diff>